<commit_message>
cleaned repo +fixed gitignore and removed useless files, promptabalations running, hybrid done.
Add script to generate numbers_master.csv from raw data sources

- Implemented a new Python script `generate_numbers_master.py` to compile metrics from various sources into a consolidated CSV file.
- The script processes per-run metrics for multiple models, computes various statistical measures, and handles RAG ablation data.
- Added functionality to calculate costs per run based on token usage and model specifications.
- Included robustness comparison between method A and imputed values.
- The output is saved as `paper/numbers_master.csv`.
</commit_message>
<xml_diff>
--- a/Analysis/RAG_Ablation/rag_ablation_bootstrap_ci.xlsx
+++ b/Analysis/RAG_Ablation/rag_ablation_bootstrap_ci.xlsx
@@ -460,13 +460,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.3256545778684238</v>
+        <v>0.2466139836730987</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2075491240871846</v>
+        <v>0.1656649758247276</v>
       </c>
       <c r="E2" t="n">
-        <v>0.4431605730722607</v>
+        <v>0.3240550350153702</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -486,13 +486,13 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.3159370989640887</v>
+        <v>0.2757061925995437</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2028985507246377</v>
+        <v>0.1939203993007504</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4262064969632444</v>
+        <v>0.3561293710362565</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -512,13 +512,13 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1087540930495027</v>
+        <v>0.06831302849881668</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.007906274145351338</v>
+        <v>-0.01052352540342323</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2191169040536979</v>
+        <v>0.1493017670003281</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -538,13 +538,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.299872137990063</v>
+        <v>0.2790198469760696</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1814958217764944</v>
+        <v>0.1994949231688788</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4131337201244105</v>
+        <v>0.3591736250297444</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -564,13 +564,13 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>-0.03888078956798695</v>
+        <v>0.001122450160373826</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.3333333333333333</v>
+        <v>-0.1752869191630169</v>
       </c>
       <c r="E6" t="n">
-        <v>0.2611030117902092</v>
+        <v>0.1722222222222222</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -590,13 +590,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.06167510761155603</v>
+        <v>0.1206276471516558</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.05839416058394162</v>
+        <v>0.04415222706218069</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1826072844352711</v>
+        <v>0.1961007731794875</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.3636485755005238</v>
+        <v>0.241260146786492</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2495243032446883</v>
+        <v>0.159599533802982</v>
       </c>
       <c r="E8" t="n">
-        <v>0.4736828048778277</v>
+        <v>0.3254007973421639</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -642,13 +642,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.3877624423422041</v>
+        <v>0.2295533300979016</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2849933608250722</v>
+        <v>0.1464059644292729</v>
       </c>
       <c r="E9" t="n">
-        <v>0.4860837852678635</v>
+        <v>0.3107489404843378</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -668,13 +668,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.08066666666666666</v>
+        <v>0.1014228395061728</v>
       </c>
       <c r="D10" t="n">
-        <v>0.0702577380952381</v>
+        <v>0.09277552469135802</v>
       </c>
       <c r="E10" t="n">
-        <v>0.09170973214285714</v>
+        <v>0.1105248611111111</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -694,13 +694,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.08592380952380953</v>
+        <v>0.09829999999999998</v>
       </c>
       <c r="D11" t="n">
-        <v>0.07349270833333334</v>
+        <v>0.08994134259259258</v>
       </c>
       <c r="E11" t="n">
-        <v>0.09906913690476192</v>
+        <v>0.1071938888888889</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -720,13 +720,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.1418053571428571</v>
+        <v>0.146637037037037</v>
       </c>
       <c r="D12" t="n">
-        <v>0.1262938541666667</v>
+        <v>0.1361506172839506</v>
       </c>
       <c r="E12" t="n">
-        <v>0.1579161011904762</v>
+        <v>0.157760524691358</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -746,13 +746,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.08537619047619047</v>
+        <v>0.09734999999999999</v>
       </c>
       <c r="D13" t="n">
-        <v>0.07348071428571427</v>
+        <v>0.0892596450617284</v>
       </c>
       <c r="E13" t="n">
-        <v>0.09776339285714283</v>
+        <v>0.1056606790123457</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -772,13 +772,13 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.09595132275132275</v>
+        <v>0.1009487654320988</v>
       </c>
       <c r="D14" t="n">
-        <v>0.07542733465608467</v>
+        <v>0.08767002829218108</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1178050066137566</v>
+        <v>0.1152905606995884</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -798,13 +798,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.1518154761904762</v>
+        <v>0.1436111111111111</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1338416071428571</v>
+        <v>0.1328731172839506</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1701109523809524</v>
+        <v>0.1547836882716049</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -824,13 +824,13 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.09274880952380953</v>
+        <v>0.1043944444444444</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0804416369047619</v>
+        <v>0.09579194444444444</v>
       </c>
       <c r="E16" t="n">
-        <v>0.1056786011904762</v>
+        <v>0.1134031327160494</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -850,13 +850,13 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.07858214285714286</v>
+        <v>0.09127777777777776</v>
       </c>
       <c r="D17" t="n">
-        <v>0.06787464285714284</v>
+        <v>0.08379691358024691</v>
       </c>
       <c r="E17" t="n">
-        <v>0.08991333333333335</v>
+        <v>0.0990798611111111</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -876,13 +876,13 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.5642857142857143</v>
+        <v>0.4703703703703704</v>
       </c>
       <c r="D18" t="n">
-        <v>0.4785714285714286</v>
+        <v>0.4111111111111111</v>
       </c>
       <c r="E18" t="n">
-        <v>0.6428571428571429</v>
+        <v>0.5296296296296297</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -902,13 +902,13 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.5785714285714286</v>
+        <v>0.5037037037037037</v>
       </c>
       <c r="D19" t="n">
-        <v>0.5</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="E19" t="n">
-        <v>0.6571428571428571</v>
+        <v>0.562962962962963</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -928,13 +928,13 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.4214285714285714</v>
+        <v>0.3888888888888889</v>
       </c>
       <c r="D20" t="n">
-        <v>0.3428571428571429</v>
+        <v>0.3296296296296296</v>
       </c>
       <c r="E20" t="n">
-        <v>0.5071428571428571</v>
+        <v>0.4481481481481481</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -954,13 +954,13 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.5428571428571428</v>
+        <v>0.5</v>
       </c>
       <c r="D21" t="n">
-        <v>0.4571428571428571</v>
+        <v>0.4407407407407408</v>
       </c>
       <c r="E21" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.5592592592592592</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -980,13 +980,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.4571428571428571</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="D22" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3444444444444444</v>
       </c>
       <c r="E22" t="n">
-        <v>0.6285714285714286</v>
+        <v>0.5444444444444444</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1006,13 +1006,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.4071428571428571</v>
+        <v>0.4370370370370371</v>
       </c>
       <c r="D23" t="n">
-        <v>0.3285714285714286</v>
+        <v>0.3777777777777778</v>
       </c>
       <c r="E23" t="n">
-        <v>0.4928571428571429</v>
+        <v>0.4962962962962963</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1032,13 +1032,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.5857142857142857</v>
+        <v>0.4888888888888889</v>
       </c>
       <c r="D24" t="n">
-        <v>0.5</v>
+        <v>0.4296296296296296</v>
       </c>
       <c r="E24" t="n">
-        <v>0.6714285714285714</v>
+        <v>0.5481481481481482</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1058,13 +1058,13 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.55</v>
+        <v>0.4666666666666667</v>
       </c>
       <c r="D25" t="n">
-        <v>0.4642857142857143</v>
+        <v>0.4074074074074074</v>
       </c>
       <c r="E25" t="n">
-        <v>0.6357142857142857</v>
+        <v>0.5259259259259259</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>

</xml_diff>